<commit_message>
Harden line-following control loop in final firmware
Fix steering D-term spike on line re-acquisition, ramp speed back up
gradually after a lost-line slowdown/stop instead of snapping to target,
and add an edge-separation sanity check to detectLine() to reject
mismatched edge pairs from unrelated features.
</commit_message>
<xml_diff>
--- a/data/inductor scaling.xlsx
+++ b/data/inductor scaling.xlsx
@@ -3,6 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="153222"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Charles\Desktop\natcar\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
   </bookViews>

</xml_diff>